<commit_message>
Edit text in JN. Add new INN in bd
</commit_message>
<xml_diff>
--- a/data/list_of_companies.xlsx
+++ b/data/list_of_companies.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="115">
   <si>
     <t>Название компании</t>
   </si>
@@ -95,21 +95,36 @@
     <t>АО «Сбербанк КИБ»</t>
   </si>
   <si>
+    <t>Инветиционный бизнес</t>
+  </si>
+  <si>
     <t>ООО НКО «ЮМани»</t>
   </si>
   <si>
+    <t>Оналйн платежи. Оплата</t>
+  </si>
+  <si>
     <t xml:space="preserve">ООО «Сбер Бизнес Софт» </t>
   </si>
   <si>
     <t>Цифровая экосистема и ИТ</t>
   </si>
   <si>
+    <t>Автоматизация бизнес процессов</t>
+  </si>
+  <si>
     <t>ООО «Сбер2В»</t>
   </si>
   <si>
+    <t>Закупки между бизнесами</t>
+  </si>
+  <si>
     <t>ООО «Цифровые Решения Регионов»</t>
   </si>
   <si>
+    <t>Технологические платформы для государства</t>
+  </si>
+  <si>
     <t>ООО «РДВ-софт»</t>
   </si>
   <si>
@@ -125,6 +140,9 @@
     <t>ООО «ЗВУК БИЗНЕС»</t>
   </si>
   <si>
+    <t>Предоставление музыки комм. помещениям</t>
+  </si>
+  <si>
     <t xml:space="preserve">ООО «Облачные технологии» </t>
   </si>
   <si>
@@ -191,6 +209,12 @@
     <t>Платформа для малого и микробизнеса</t>
   </si>
   <si>
+    <t>ООО «Сбербанк-Телеком»</t>
+  </si>
+  <si>
+    <t>Оператор связи</t>
+  </si>
+  <si>
     <t>ООО «Умный ритейл» (Самокат)</t>
   </si>
   <si>
@@ -212,7 +236,7 @@
     <t>Медицина</t>
   </si>
   <si>
-    <t>Онлайн-аптека и заказ медикаментов</t>
+    <t>Онлайн-аптека и заказ медикаментов (во владении 45%)</t>
   </si>
   <si>
     <t>ООО «ДокДок Территория Здоровья»</t>
@@ -246,6 +270,30 @@
   </si>
   <si>
     <t>Строительство недвижемости</t>
+  </si>
+  <si>
+    <t>ООО «СберАвто»</t>
+  </si>
+  <si>
+    <t>Авто</t>
+  </si>
+  <si>
+    <t>Платформа для покупки, продажи и обслуживания автомобилей онлайн.</t>
+  </si>
+  <si>
+    <t>ООО «Сити Драйв»</t>
+  </si>
+  <si>
+    <t>Каршеринг</t>
+  </si>
+  <si>
+    <t>АНО «Корпоративный университет Сбербанка»</t>
+  </si>
+  <si>
+    <t>Образование</t>
+  </si>
+  <si>
+    <t>Дополнительно образование для сотруников</t>
   </si>
   <si>
     <t>ПАО «Сегежа Групп»</t>
@@ -347,14 +395,14 @@
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="10.0"/>
-      <color rgb="FF26364B"/>
+      <color theme="1"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="10.0"/>
       <color rgb="FF26364B"/>
-      <name val="Inter"/>
+      <name val="Arial"/>
     </font>
     <font>
       <sz val="10.0"/>
@@ -417,7 +465,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -425,8 +473,14 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="2" fontId="5" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -845,68 +899,78 @@
       <c r="B12" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="2"/>
+      <c r="C12" s="5" t="s">
+        <v>27</v>
+      </c>
       <c r="D12" s="2">
         <v>7.71004897E9</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C13" s="2"/>
+      <c r="C13" s="5" t="s">
+        <v>29</v>
+      </c>
       <c r="D13" s="2">
         <v>7.750005725E9</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C14" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>32</v>
+      </c>
       <c r="D14" s="2">
         <v>7.73026955E9</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C15" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>34</v>
+      </c>
       <c r="D15" s="2">
         <v>7.730241227E9</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C16" s="2"/>
+      <c r="C16" s="5" t="s">
+        <v>36</v>
+      </c>
       <c r="D16" s="2">
         <v>7.730261382E9</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D17" s="2">
         <v>7.707083893E9</v>
@@ -914,13 +978,13 @@
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D18" s="2">
         <v>7.708328948E9</v>
@@ -928,25 +992,27 @@
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C19" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="D19" s="2">
         <v>7.801445445E9</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="4" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D20" s="2">
         <v>7.73627916E9</v>
@@ -954,13 +1020,13 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D21" s="2">
         <v>7.73025372E9</v>
@@ -968,13 +1034,13 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="D22" s="2">
         <v>9.73105395E9</v>
@@ -982,27 +1048,27 @@
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D23" s="5">
+        <v>50</v>
+      </c>
+      <c r="D23" s="6">
         <v>7.736319695E9</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="D24" s="2">
         <v>7.801392271E9</v>
@@ -1010,13 +1076,13 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="D25" s="2">
         <v>5.405276231E9</v>
@@ -1024,13 +1090,13 @@
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="D26" s="2">
         <v>7.710561081E9</v>
@@ -1038,13 +1104,13 @@
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D27" s="2">
         <v>7.70730848E9</v>
@@ -1052,13 +1118,13 @@
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="D28" s="2">
         <v>7.736632467E9</v>
@@ -1066,13 +1132,13 @@
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D29" s="2">
         <v>7.736663049E9</v>
@@ -1080,156 +1146,208 @@
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D30" s="2">
         <v>7.736641983E9</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="2" t="s">
-        <v>59</v>
+      <c r="A31" s="7" t="s">
+        <v>65</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="D31" s="2">
-        <v>7.811657093E9</v>
+        <v>31</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D31" s="7">
+        <v>7.736264044E9</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="D32" s="2">
-        <v>9.705118142E9</v>
+        <v>7.811657093E9</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="D33" s="2">
+        <v>9.705118142E9</v>
+      </c>
+    </row>
+    <row r="34" ht="15.75" customHeight="1">
+      <c r="A34" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D34" s="2">
         <v>7.70486554E9</v>
       </c>
     </row>
-    <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="D34" s="7">
+    <row r="35" ht="15.75" customHeight="1">
+      <c r="A35" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D35" s="9">
         <v>9.71004992E9</v>
       </c>
     </row>
-    <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D35" s="2">
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="A36" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D36" s="2">
         <v>7.714427506E9</v>
       </c>
     </row>
-    <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="D36" s="8">
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="A37" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D37" s="10">
         <v>9.70512494E9</v>
       </c>
     </row>
-    <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="D37" s="2">
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="A38" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D38" s="2">
         <v>5.024093941E9</v>
       </c>
     </row>
-    <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="B38" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="C38" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="D38" s="9">
+    <row r="39" ht="15.75" customHeight="1">
+      <c r="A39" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="D39" s="7">
+        <v>9.709054813E9</v>
+      </c>
+    </row>
+    <row r="40" ht="15.75" customHeight="1">
+      <c r="A40" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D40" s="7">
+        <v>7.727833329E9</v>
+      </c>
+    </row>
+    <row r="41" ht="15.75" customHeight="1">
+      <c r="A41" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="D41" s="7">
+        <v>7.736128605E9</v>
+      </c>
+    </row>
+    <row r="42" ht="15.75" customHeight="1">
+      <c r="A42" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="B42" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="C42" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="D42" s="11">
         <v>9.703024202E9</v>
       </c>
-      <c r="E38" s="9"/>
-      <c r="F38" s="9"/>
-      <c r="G38" s="9"/>
-      <c r="H38" s="9"/>
-      <c r="I38" s="9"/>
-      <c r="J38" s="9"/>
-      <c r="K38" s="9"/>
-      <c r="L38" s="9"/>
-      <c r="M38" s="9"/>
-      <c r="N38" s="9"/>
-      <c r="O38" s="9"/>
-      <c r="P38" s="9"/>
-      <c r="Q38" s="9"/>
-      <c r="R38" s="9"/>
-      <c r="S38" s="9"/>
-      <c r="T38" s="9"/>
-      <c r="U38" s="9"/>
-      <c r="V38" s="9"/>
-      <c r="W38" s="9"/>
-      <c r="X38" s="9"/>
-      <c r="Y38" s="9"/>
-      <c r="Z38" s="9"/>
-    </row>
-    <row r="39" ht="15.75" customHeight="1"/>
-    <row r="40" ht="15.75" customHeight="1"/>
-    <row r="41" ht="15.75" customHeight="1"/>
-    <row r="42" ht="15.75" customHeight="1"/>
+      <c r="E42" s="11"/>
+      <c r="F42" s="11"/>
+      <c r="G42" s="11"/>
+      <c r="H42" s="11"/>
+      <c r="I42" s="11"/>
+      <c r="J42" s="11"/>
+      <c r="K42" s="11"/>
+      <c r="L42" s="11"/>
+      <c r="M42" s="11"/>
+      <c r="N42" s="11"/>
+      <c r="O42" s="11"/>
+      <c r="P42" s="11"/>
+      <c r="Q42" s="11"/>
+      <c r="R42" s="11"/>
+      <c r="S42" s="11"/>
+      <c r="T42" s="11"/>
+      <c r="U42" s="11"/>
+      <c r="V42" s="11"/>
+      <c r="W42" s="11"/>
+      <c r="X42" s="11"/>
+      <c r="Y42" s="11"/>
+      <c r="Z42" s="11"/>
+    </row>
     <row r="43" ht="15.75" customHeight="1"/>
     <row r="44" ht="15.75" customHeight="1"/>
     <row r="45" ht="15.75" customHeight="1"/>
@@ -2188,6 +2306,10 @@
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
+    <row r="1001" ht="15.75" customHeight="1"/>
+    <row r="1002" ht="15.75" customHeight="1"/>
+    <row r="1003" ht="15.75" customHeight="1"/>
+    <row r="1004" ht="15.75" customHeight="1"/>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -2212,34 +2334,34 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="11" t="s">
-        <v>81</v>
+      <c r="A1" s="13" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
-      <c r="A2" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="B2" s="12" t="s">
+      <c r="A2" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="B2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="E2" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="F2" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="G2" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="H2" s="13" t="s">
-        <v>87</v>
+      <c r="D2" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="F2" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="G2" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
@@ -2252,14 +2374,14 @@
       <c r="C3" s="2">
         <v>7.707009586E9</v>
       </c>
-      <c r="D3" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="E3" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>90</v>
+      <c r="D3" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="E3" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>106</v>
       </c>
       <c r="G3" s="2">
         <v>701.0</v>
@@ -2267,7 +2389,7 @@
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2">
@@ -2281,12 +2403,12 @@
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C5" s="5">
+        <v>107</v>
+      </c>
+      <c r="C5" s="6">
         <v>7.736319695E9</v>
       </c>
       <c r="G5" s="2">
@@ -2295,10 +2417,10 @@
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="C6" s="2">
         <v>7.736632467E9</v>
@@ -2309,10 +2431,10 @@
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="C7" s="2">
         <v>7.736663049E9</v>
@@ -2323,10 +2445,10 @@
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="C8" s="2">
         <v>7.736641983E9</v>
@@ -2337,10 +2459,10 @@
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="C9" s="2">
         <v>7.710561081E9</v>
@@ -2351,10 +2473,10 @@
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="C10" s="2">
         <v>7.73627916E9</v>
@@ -2365,10 +2487,10 @@
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="C11" s="2">
         <v>7.73025372E9</v>
@@ -2379,10 +2501,10 @@
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="C12" s="2">
         <v>7.708328948E9</v>
@@ -2392,58 +2514,58 @@
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="D13" s="15"/>
+      <c r="D13" s="17"/>
       <c r="G13" s="2"/>
     </row>
     <row r="14" ht="15.75" customHeight="1"/>
     <row r="15" ht="15.75" customHeight="1">
-      <c r="A15" s="17" t="s">
-        <v>93</v>
+      <c r="A15" s="19" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
-      <c r="A16" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="B16" s="12" t="s">
+      <c r="A16" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="B16" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C16" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="D16" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="E16" s="13" t="s">
-        <v>94</v>
-      </c>
-      <c r="F16" s="13"/>
+      <c r="D16" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="F16" s="15"/>
       <c r="I16" s="2"/>
-      <c r="K16" s="13"/>
+      <c r="K16" s="15"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="C17" s="2">
         <v>7.811657093E9</v>
       </c>
-      <c r="D17" s="15" t="s">
-        <v>96</v>
-      </c>
-      <c r="E17" s="15" t="s">
-        <v>97</v>
+      <c r="D17" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="E17" s="17" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="C18" s="2">
         <v>9.705118142E9</v>
@@ -2451,32 +2573,32 @@
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="C19" s="2">
         <v>7.70486554E9</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="6" t="s">
-        <v>67</v>
+      <c r="A20" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C20" s="18">
+        <v>73</v>
+      </c>
+      <c r="C20" s="20">
         <v>9.71004992E9</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="C21" s="2">
         <v>7.714427506E9</v>

</xml_diff>